<commit_message>
Exam duty: swap Warin (Wed 28 Oct evening) with Pornchanok (Sat 31 Oct evening) via changes.json
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FapC72tTBB8AqE8phsKq6c
</commit_message>
<xml_diff>
--- a/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
+++ b/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ร่างตารางคุมสอบ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ร่างตารางคุมสอบ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อรชร - วรินทร, กชกานต์</t>
+          <t>ผศ.ดร.อรชร - พรชนก, กชกานต์</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อัจฉรา - พรชนก</t>
+          <t>ผศ.ดร.อัจฉรา - วรินทร</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Exam duty: apply 35 replacement requests from the change forms (changes.json replace), clash check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FapC72tTBB8AqE8phsKq6c
</commit_message>
<xml_diff>
--- a/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
+++ b/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
@@ -769,12 +769,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ปราน - สิรินภัทร, วชิรวิทย์</t>
+          <t>อ.ดร.ปราน - สิรินภัทร, กชกานต์</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ไกรวุฒิ - สัพพัญญู</t>
+          <t>ผศ.ดร.ไกรวุฒิ - อติกานต์</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วันพัฒน์ - รัชนีวรรณ, อติกานต์</t>
+          <t>ผศ.ดร.วันพัฒน์ - อิสรีย์, อติกานต์</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.พรชนก - อารยา, วรินทร</t>
+          <t>อ.ดร.พรชนก - สกาวกวิน, วรินทร</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>ฐิตารีย์, รัชนีวรรณ</t>
+          <t>ฐิตารีย์, วีรภัทร์</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ราม - สัพพัญญู, อิสรีย์</t>
+          <t>ผศ.ราม - พีชชา, อิสรีย์</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>อ.ณิศนีญ์ - สุภีฤทัย</t>
+          <t>อ.ณิศนีญ์ - วรินทร</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐกร - สิรินภัทร, ภัทรลภา, ณภัคสุรางค์</t>
+          <t>ผศ.ดร.ณัฐกร - สิรินภัทร, ภัทรลภา, สกาวกวิน</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>อ.ณิศนีญ์ - สุภีฤทัย</t>
+          <t>อ.ณิศนีญ์ - วรินทร</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1849,12 +1849,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ปราน - กชกานต์</t>
+          <t>อ.ดร.ปราน - อารยา</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ภาณุวัฒน์ - วชิราวุธ</t>
+          <t>ผศ.ดร.ภาณุวัฒน์ - ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1954,12 +1954,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ธันยวัฒน์ - พรชนก</t>
+          <t>รศ.ดร.ธันยวัฒน์ - ภัทรลภา</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วรพงศ์ - ณัฏฐพัชร</t>
+          <t>ผศ.ดร.วรพงศ์ - ธีราภัณฑ์</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>ภัทรลภา - ชนะชล</t>
+          <t>มาธวี - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ภาณุวัฒน์ - ลัดดาภรณ์</t>
+          <t>ผศ.ดร.ภาณุวัฒน์ - วีรภัทร์</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>ภัทรลภา - ชนะชล</t>
+          <t>มาธวี - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.พจนา - พิชชารีย์</t>
+          <t>ผศ.ดร.พจนา - วีรภัทร์</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.รวีวรรณ - สกาวกวิน</t>
+          <t>ผศ.ดร.รวีวรรณ - อารยา</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วรรณภา - ณภัคสุรางค์, สิรินภัทร</t>
+          <t>ผศ.ดร.วรรณภา - ธีราภัณฑ์, สิรินภัทร</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐพล - วชิรวิทย์, ณัฐธยาน์</t>
+          <t>ผศ.ดร.ณัฐพล - มาธวี, ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วรพงศ์ - สัพพัญญู</t>
+          <t>ผศ.ดร.วรพงศ์ - กชกานต์</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -2454,12 +2454,12 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อัจฉรียา - โศศิษฐา</t>
+          <t>ผศ.ดร.อัจฉรียา - พีชชา</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศิรดา - สุภีฤทัย</t>
+          <t>อ.ดร.ศิรดา - วชิรวิทย์</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>รุ่งทิวา - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.Matthew - รัชนีวรรณ</t>
+          <t>อ.ดร.Matthew - ภัทรลภา</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.เบญจมาศ - สุภีฤทัย</t>
+          <t>ผศ.ดร.เบญจมาศ - ธีราภัณฑ์</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.รวีวรรณ - ณัฏฐพัชร</t>
+          <t>ผศ.ดร.รวีวรรณ - ชัยตรี</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อรชร - พรชนก, กชกานต์</t>
+          <t>ผศ.ดร.อรชร - วรินทร, วชิรวิทย์</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐกร - อารยา, สัพพัญญู</t>
+          <t>ผศ.ดร.ณัฐกร - อารยา, วรินทร</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วันพัฒน์ - วชิราวุธ</t>
+          <t>ผศ.ดร.วันพัฒน์ - มาธวี</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="G116" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศิรดา - รัชนีวรรณ</t>
+          <t>อ.ดร.ศิรดา - วีรภัทร์</t>
         </is>
       </c>
       <c r="G118" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="G120" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.พินสุดา - ลัดดาภรณ์</t>
+          <t>อ.ดร.พินสุดา - วรินทร</t>
         </is>
       </c>
       <c r="G126" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Exam duty: add 127303 (21 Oct, PSB1205/1206), move Phitcha to PSB1306 and Sakaokawin to PSB1312
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FapC72tTBB8AqE8phsKq6c
</commit_message>
<xml_diff>
--- a/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
+++ b/exam-duty-dashboard/ร่างตารางคุมสอบ_1-2569.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,13 +40,9 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009C0006"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +57,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCE6F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -112,10 +103,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -484,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -821,7 +809,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>127428</t>
+          <t>127303</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -831,15 +819,15 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1205</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.มาลินี - มาธวี</t>
+          <t>อ.ดร.พินสุดา - โศศิษฐา</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -856,7 +844,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>128202</t>
+          <t>127303</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -866,15 +854,15 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>PSB1201</t>
+          <t>PSB1206</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ปฐมาวดี - ภัทรลภา</t>
+          <t>ธนภัทร, สิริมา</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -891,25 +879,25 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>128202</t>
+          <t>127428</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>PSB1310</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศศิพัชร์ - ชัยตรี</t>
+          <t>ผศ.ดร.มาลินี - มาธวี</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -926,145 +914,145 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>128202</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>PSB1201</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>รศ.ดร.ปฐมาวดี - ภัทรลภา</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>128202</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>PSB1310</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>อ.ดร.ศศิพัชร์ - ชัยตรี</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>128434</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>PSB1307</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E19" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>ผศ.ดร.ไกรวุฒิ - อติกานต์</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>วันพฤหัสบดีที่ 22 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>126346</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>PSB1201</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.พิชญ์อาภา - ภูษณิศา</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>127202</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>PSB1101</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>77</v>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.วันพัฒน์ - อิสรีย์, อติกานต์</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1064,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>127327</t>
+          <t>126346</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1086,15 +1074,15 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1201</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.สุพิชฌาย์ - รุ่งทิวา</t>
+          <t>ผศ.ดร.พิชญ์อาภา - ภูษณิศา</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1111,7 +1099,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>127416</t>
+          <t>127202</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1121,15 +1109,15 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.พรชนก - วรินทร</t>
+          <t>ผศ.ดร.วันพัฒน์ - อิสรีย์, อติกานต์</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1146,7 +1134,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>127711</t>
+          <t>127327</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1156,15 +1144,15 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>PSB1303</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.มาลินี</t>
+          <t>ผศ.ดร.สุพิชฌาย์ - รุ่งทิวา</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1181,7 +1169,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>128334</t>
+          <t>127416</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1191,15 +1179,15 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>PSB1208</t>
+          <t>AUD50</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ไกรวุฒิ - กชกานต์</t>
+          <t>อ.ดร.พรชนก - วรินทร</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1216,7 +1204,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>128425</t>
+          <t>127711</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1226,15 +1214,15 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>PSB1303</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>รศ.ศิริพงษ์ - วชิราวุธ</t>
+          <t>ผศ.ดร.มาลินี</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1251,25 +1239,25 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>213362</t>
+          <t>128334</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>PSB1302</t>
+          <t>PSB1208</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>อ.ภูมิศร์</t>
+          <t>ผศ.ดร.ไกรวุฒิ - กชกานต์</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1286,25 +1274,25 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>213362</t>
+          <t>128425</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>702</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>PSB1302</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>อ.ภูมิศร์</t>
+          <t>รศ.ศิริพงษ์ - วชิราวุธ</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1316,162 +1304,162 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>213362</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>PSB1302</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>อ.ภูมิศร์</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>พีชชา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>213362</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>PSB1302</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>อ.ภูมิศร์</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>พีชชา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
           <t>13:00-16:00</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>127759</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>PSB1306</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E31" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>รศ.ดร.ธัญณ์ณภัทร์</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>มาธวี - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>วันเสาร์ที่ 24 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>12:00-13:30</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>127100</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>PSB1101</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>135</v>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.พรชนก - สกาวกวิน, วรินทร</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ชนะชล</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>15:30-18:30</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>127101</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>PSB1204</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>ฐิตารีย์, วีรภัทร์</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>วชิรวิทย์ - ชนะชล</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>12:00-13:30</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>127101</t>
+          <t>127100</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1481,20 +1469,20 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>PSB1205</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>40</v>
+        <v>135</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.พินสุดา - ชัยตรี</t>
+          <t>อ.ดร.พรชนก - สกาวกวิน, วรินทร</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>วชิรวิทย์ - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1511,20 +1499,20 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>PSB1101</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>122</v>
+        <v>37</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ราม - พีชชา, อิสรีย์</t>
+          <t>ฐิตารีย์, วีรภัทร์</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -1546,20 +1534,20 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>PSB1201</t>
+          <t>PSB1205</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>วริชา, ณัฐธยาน์</t>
+          <t>อ.ดร.พินสุดา - ชัยตรี</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -1581,20 +1569,20 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>PSB1310</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>อ.ณิศนีญ์ - วรินทร</t>
+          <t>ผศ.ราม - พีชชา, อิสรีย์</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -1616,20 +1604,20 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>002</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1201</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>169</v>
+        <v>39</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐกร - สิรินภัทร, ภัทรลภา, สกาวกวิน</t>
+          <t>วริชา, ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -1651,140 +1639,140 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>PSB1310</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>อ.ณิศนีญ์ - วรินทร</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์ - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>127101</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>AUD50</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>169</v>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.ณัฐกร - สิรินภัทร, ภัทรลภา, สกาวกวิน</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์ - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>127101</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
           <t>701</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>PSB1310</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E41" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>อ.ณิศนีญ์ - วรินทร</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>วชิรวิทย์ - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>วันอาทิตย์ที่ 25 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>126216</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>PSB1205</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.Matthew - อติกานต์</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ชนะชล</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>126216</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>PSB1208</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.อัจฉรียา - พีชชา</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -1801,20 +1789,20 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>PSB1312</t>
+          <t>PSB1205</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.กมลพร - ภูษณิศา</t>
+          <t>อ.ดร.Matthew - อติกานต์</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -1836,20 +1824,20 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>002</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>PSB1311</t>
+          <t>PSB1208</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ปราน - อารยา</t>
+          <t>ผศ.ดร.อัจฉรียา - พีชชา</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -1866,25 +1854,25 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>126338</t>
+          <t>126216</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>PSB1312</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.เบญจมาศ - สารัตถ์</t>
+          <t>ผศ.ดร.กมลพร - ภูษณิศา</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -1901,25 +1889,25 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>127411</t>
+          <t>126216</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>004</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>PSB1101</t>
+          <t>PSB1311</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ภาณุวัฒน์ - ณัฐธยาน์</t>
+          <t>อ.ดร.ปราน - อารยา</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -1936,7 +1924,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>128204</t>
+          <t>126338</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -1946,15 +1934,15 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>PSB1307</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ธันยวัฒน์ - ภัทรลภา</t>
+          <t>ผศ.ดร.เบญจมาศ - สารัตถ์</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -1971,25 +1959,25 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>128204</t>
+          <t>127411</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.พนม - วีรภัทร์</t>
+          <t>ผศ.ดร.ภาณุวัฒน์ - ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2006,7 +1994,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>128354</t>
+          <t>128204</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -2016,15 +2004,15 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1307</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วรพงศ์ - ธีราภัณฑ์</t>
+          <t>รศ.ดร.ธันยวัฒน์ - ภัทรลภา</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -2041,25 +2029,25 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>128357</t>
+          <t>128204</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>PSB1206</t>
+          <t>AUD50</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ฐิติวุฒิ - สิริมา</t>
+          <t>รศ.ดร.พนม - วีรภัทร์</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -2071,12 +2059,12 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>12:00-15:00</t>
+          <t>08:00-11:00</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>127717</t>
+          <t>128354</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -2086,67 +2074,67 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>PSB1303</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐพล</t>
+          <t>ผศ.ดร.วรพงศ์ - ธีราภัณฑ์</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>มาธวี - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>12:00-15:00</t>
+          <t>08:00-11:00</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>127717</t>
+          <t>128357</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>801</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1206</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ภาณุวัฒน์ - วีรภัทร์</t>
+          <t>รศ.ดร.ฐิติวุฒิ - สิริมา</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>มาธวี - ชนะชล</t>
+          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>12:00-15:00</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>128307</t>
+          <t>127717</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -2156,15 +2144,15 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>PSB1205</t>
+          <t>PSB1303</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.พจนา - วีรภัทร์</t>
+          <t>ผศ.ดร.ณัฐพล</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2176,150 +2164,150 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>127717</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>801</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>PSB1207</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.ภาณุวัฒน์ - วีรภัทร์</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>มาธวี - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
           <t>15:30-18:30</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>128307</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>PSB1205</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.พจนา - วีรภัทร์</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>มาธวี - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>128307</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>PSB1204</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E57" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>ผศ.ดร.รวีวรรณ - อารยา</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>มาธวี - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>วันจันทร์ที่ 26 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>126321</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>PSB1101</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="n">
-        <v>98</v>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.วรรณภา - ธีราภัณฑ์, สิรินภัทร</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ชนะชล</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>126324</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>PSB1207</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.กัญญณัฏฐา - ธนภัทร</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2319,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>127316</t>
+          <t>126321</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -2341,15 +2329,15 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ณัฐพล - มาธวี, ณัฐธยาน์</t>
+          <t>ผศ.ดร.วรรณภา - ธีราภัณฑ์, สิรินภัทร</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -2366,7 +2354,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>128431</t>
+          <t>126324</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -2376,15 +2364,15 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>PSB1307</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.วรพงศ์ - กชกานต์</t>
+          <t>ผศ.ดร.กัญญณัฏฐา - ธนภัทร</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -2401,25 +2389,25 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>131201</t>
+          <t>127316</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>AUD50</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.เบญจมาศ - ชัยตรี</t>
+          <t>ผศ.ดร.ณัฐพล - มาธวี, ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
@@ -2431,12 +2419,12 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>08:00-11:00</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>126339</t>
+          <t>128431</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -2446,15 +2434,15 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1307</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อัจฉรียา - พีชชา</t>
+          <t>ผศ.ดร.วรพงศ์ - กชกานต์</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
@@ -2466,17 +2454,17 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>08:00-11:00</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>126341</t>
+          <t>131201</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>701</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2489,7 +2477,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศิรดา - วชิรวิทย์</t>
+          <t>ผศ.ดร.เบญจมาศ - ชัยตรี</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -2506,7 +2494,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>126348</t>
+          <t>126339</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2516,15 +2504,15 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>PSB1208</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.Matthew - วริชา</t>
+          <t>ผศ.ดร.อัจฉรียา - พีชชา</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
@@ -2541,25 +2529,25 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>126348</t>
+          <t>126341</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>PSB1208</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.Matthew - วริชา</t>
+          <t>อ.ดร.ศิรดา - วชิรวิทย์</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
@@ -2576,7 +2564,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>127312</t>
+          <t>126348</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -2586,15 +2574,15 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>PSB1101</t>
+          <t>PSB1208</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>121</v>
+        <v>10</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.มาลินี - ฐิตารีย์, อารยา</t>
+          <t>อ.ดร.Matthew - วริชา</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
@@ -2611,157 +2599,157 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
+          <t>126348</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>PSB1208</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>อ.ดร.Matthew - วริชา</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>127312</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>PSB1101</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.มาลินี - ฐิตารีย์, อารยา</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
           <t>127417</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>AUD50</t>
         </is>
       </c>
-      <c r="E68" s="4" t="n">
+      <c r="E70" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="F68" s="5" t="inlineStr">
+      <c r="F70" s="5" t="inlineStr">
         <is>
           <t>ผศ.ราม - อิสรีย์</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>วรินทร - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>วันอังคารที่ 27 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>128427</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>PSB1307</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.นัทธพงศ์ - ภัทรลภา</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr">
-        <is>
-          <t>ภัทรลภา - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>126101</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>PSB1308</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.ปราน - ณัฐธยาน์</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>อติกานต์ - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>12:00-15:00</t>
+          <t>08:00-11:00</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>126101</t>
+          <t>128427</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -2771,20 +2759,20 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>PSB1309</t>
+          <t>PSB1307</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>มาธวี, พิชชารีย์</t>
+          <t>อ.ดร.นัทธพงศ์ - ภัทรลภา</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>อติกานต์ - ธีราภัณฑ์</t>
+          <t>ภัทรลภา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -2801,20 +2789,20 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1308</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อัจฉรา - วีรภัทร์, กชกานต์</t>
+          <t>อ.ดร.ปราน - ณัฐธยาน์</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -2836,20 +2824,20 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>PSB1201</t>
+          <t>PSB1309</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.พิชญ์อาภา - โศศิษฐา</t>
+          <t>มาธวี, พิชชารีย์</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -2871,20 +2859,20 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>AUD50</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>ณัฏฐพัชร, อิสรีย์</t>
+          <t>ผศ.ดร.อัจฉรา - วีรภัทร์, กชกานต์</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -2906,20 +2894,20 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1201</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.พฤดี - สัพพัญญู</t>
+          <t>ผศ.ดร.พิชญ์อาภา - โศศิษฐา</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -2941,20 +2929,20 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>PSB1306</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>⚠ ยังขาดคนคุม</t>
+        <v>34</v>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>ณัฏฐพัชร, อิสรีย์</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -2981,7 +2969,7 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>PSB1311</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
@@ -2989,7 +2977,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>อารยา, วริชา</t>
+          <t>รศ.ดร.พฤดี - สัพพัญญู</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -3016,15 +3004,15 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>PSB1312</t>
+          <t>PSB1306</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>ชัยตรี, พีชชา</t>
+          <t>พีชชา</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -3046,20 +3034,20 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>PSB1307</t>
+          <t>PSB1311</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>สิรินภัทร, วชิรวิทย์</t>
+          <t>อารยา, วริชา</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -3081,20 +3069,20 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>PSB1310</t>
+          <t>PSB1312</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.อัจฉรียา - รุ่งทิวา</t>
+          <t>สกาวกวิน, ชัยตรี</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3116,20 +3104,20 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>006</t>
+          <t>005</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>PSB1205</t>
+          <t>PSB1307</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.กัญญณัฏฐา - ธนภัทร</t>
+          <t>สิรินภัทร, วชิรวิทย์</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -3151,20 +3139,20 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>006</t>
+          <t>005</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>PSB1206</t>
+          <t>PSB1310</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>วชิราวุธ, ลัดดาภรณ์</t>
+          <t>ผศ.ดร.อัจฉรียา - รุ่งทิวา</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -3186,20 +3174,20 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>006</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>PSB1208</t>
+          <t>PSB1205</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>ฐิตารีย์, ณภัคสุรางค์</t>
+          <t>ผศ.ดร.กัญญณัฏฐา - ธนภัทร</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -3221,20 +3209,20 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>006</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>PSB1302</t>
+          <t>PSB1206</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศิรดา - วรินทร</t>
+          <t>วชิราวุธ, ลัดดาภรณ์</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -3261,15 +3249,15 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>PSB1303</t>
+          <t>PSB1208</t>
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>สุภีฤทัย</t>
+          <t>ฐิตารีย์, ณภัคสุรางค์</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -3291,25 +3279,25 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>007</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>ECON-A</t>
+          <t>PSB1302</t>
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.Matthew - ภัทรลภา</t>
+          <t>อ.ดร.ศิรดา - วรินทร</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>อติกานต์ - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -3326,25 +3314,25 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>702</t>
+          <t>007</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>ECON-B</t>
+          <t>PSB1303</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.LEE - สารัตถ์, สกาวกวิน</t>
+          <t>สุภีฤทัย</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>พรชนก - ธีราภัณฑ์</t>
+          <t>อติกานต์ - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -3356,145 +3344,145 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
+          <t>126101</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>ECON-A</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>อ.ดร.Matthew - ภัทรลภา</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>พรชนก - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>126101</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>ECON-B</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>รศ.ดร.LEE - สารัตถ์</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>พรชนก - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
           <t>128203</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
         <is>
           <t>PSB1101</t>
         </is>
       </c>
-      <c r="E90" s="4" t="n">
+      <c r="E92" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="F90" s="5" t="inlineStr">
+      <c r="F92" s="5" t="inlineStr">
         <is>
           <t>อ.ดร.นัทธพงศ์ - สิริมา, ภูษณิศา</t>
         </is>
       </c>
-      <c r="G90" s="5" t="inlineStr">
+      <c r="G92" s="5" t="inlineStr">
         <is>
           <t>อติกานต์ - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="A91" s="2" t="inlineStr">
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>วันพุธที่ 28 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="30" customHeight="1">
-      <c r="A92" s="3" t="inlineStr">
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr">
+      <c r="B94" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C92" s="3" t="inlineStr">
+      <c r="C94" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D92" s="3" t="inlineStr">
+      <c r="D94" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr">
+      <c r="E94" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F92" s="3" t="inlineStr">
+      <c r="F94" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G92" s="3" t="inlineStr">
+      <c r="G94" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>126427</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>PSB1307</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.เบญจมาศ - ธีราภัณฑ์</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ชนะชล</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>126460</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>PSB1204</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.กมลพร - อิสรีย์</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3494,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>128355</t>
+          <t>126427</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -3516,15 +3504,15 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>PSB1207</t>
+          <t>PSB1307</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.พนม - สารัตถ์</t>
+          <t>ผศ.ดร.เบญจมาศ - ธีราภัณฑ์</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -3541,7 +3529,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>128462</t>
+          <t>126460</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -3551,15 +3539,15 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>PSB1208</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ฐิติวุฒิ</t>
+          <t>ผศ.ดร.กมลพร - อิสรีย์</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -3571,12 +3559,12 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>12:00-15:00</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>128101</t>
+          <t>128355</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -3586,55 +3574,55 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>PSB1207</t>
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>รศ.ศิริพงษ์ - วีรภัทร์</t>
+          <t>รศ.ดร.พนม - สารัตถ์</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>ภูษณิศา - ชนะชล</t>
+          <t>พีชชา - ชนะชล</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>15:30-18:30</t>
+          <t>12:00-15:00</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>128101</t>
+          <t>128462</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>PSB1201</t>
+          <t>PSB1208</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.รวีวรรณ - ชัยตรี</t>
+          <t>รศ.ดร.ฐิติวุฒิ</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>ภูษณิศา - ชนะชล</t>
+          <t>พีชชา - ชนะชล</t>
         </is>
       </c>
     </row>
@@ -3651,20 +3639,20 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1204</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>อ.พิกุล - สิริมา, ธนภัทร</t>
+          <t>รศ.ศิริพงษ์ - วีรภัทร์</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -3686,140 +3674,140 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>PSB1201</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.รวีวรรณ - ชัยตรี</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>ภูษณิศา - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>128101</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>AUD50</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>อ.พิกุล - สิริมา, ธนภัทร</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>ภูษณิศา - ชนะชล</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>128101</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
           <t>004</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
+      <c r="D102" s="4" t="inlineStr">
         <is>
           <t>PSB1101</t>
         </is>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E102" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="F100" s="5" t="inlineStr">
+      <c r="F102" s="5" t="inlineStr">
         <is>
           <t>ผศ.ดร.อรชร - วรินทร, วชิรวิทย์</t>
         </is>
       </c>
-      <c r="G100" s="5" t="inlineStr">
+      <c r="G102" s="5" t="inlineStr">
         <is>
           <t>ภูษณิศา - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="A101" s="2" t="inlineStr">
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>วันพฤหัสบดีที่ 29 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="30" customHeight="1">
-      <c r="A102" s="3" t="inlineStr">
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr">
+      <c r="C104" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D102" s="3" t="inlineStr">
+      <c r="D104" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E102" s="3" t="inlineStr">
+      <c r="E104" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F102" s="3" t="inlineStr">
+      <c r="F104" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G102" s="3" t="inlineStr">
+      <c r="G104" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>127317</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr">
-        <is>
-          <t>PSB1101</t>
-        </is>
-      </c>
-      <c r="E103" s="4" t="n">
-        <v>85</v>
-      </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.ณัฐกร - อารยา, วรินทร</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>รุ่งทิวา - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>128403</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>PSB1205</t>
-        </is>
-      </c>
-      <c r="E104" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="F104" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.อุดมโชค - พิชชารีย์</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>รุ่งทิวา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -3831,225 +3819,225 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
+          <t>127317</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>PSB1101</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.ณัฐกร - อารยา, วรินทร</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>รุ่งทิวา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>128403</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>PSB1205</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.อุดมโชค - พิชชารีย์</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>รุ่งทิวา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>12:00-15:00</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
           <t>131204</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
         <is>
           <t>701</t>
         </is>
       </c>
-      <c r="D105" s="4" t="inlineStr">
+      <c r="D107" s="4" t="inlineStr">
         <is>
           <t>PSB1204</t>
         </is>
       </c>
-      <c r="E105" s="4" t="n">
+      <c r="E107" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F107" s="5" t="inlineStr">
         <is>
           <t>รศ.ดร.วิชชุดา - ฐิตารีย์</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G107" s="5" t="inlineStr">
         <is>
           <t>รุ่งทิวา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="20" customHeight="1">
-      <c r="A106" s="2" t="inlineStr">
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
         <is>
           <t>วันศุกร์ที่ 30 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="30" customHeight="1">
-      <c r="A107" s="3" t="inlineStr">
+    <row r="109" ht="30" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C107" s="3" t="inlineStr">
+      <c r="C109" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D107" s="3" t="inlineStr">
+      <c r="D109" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E107" s="3" t="inlineStr">
+      <c r="E109" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F107" s="3" t="inlineStr">
+      <c r="F109" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G107" s="3" t="inlineStr">
+      <c r="G109" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="4" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>12:00-15:00</t>
         </is>
       </c>
-      <c r="B108" s="4" t="inlineStr">
+      <c r="B110" s="4" t="inlineStr">
         <is>
           <t>128324</t>
         </is>
       </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
         <is>
           <t>PSB1207</t>
         </is>
       </c>
-      <c r="E108" s="4" t="n">
+      <c r="E110" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F108" s="5" t="inlineStr">
+      <c r="F110" s="5" t="inlineStr">
         <is>
           <t>อ.ดร.นัทธพงศ์ - อติกานต์</t>
         </is>
       </c>
-      <c r="G108" s="5" t="inlineStr">
+      <c r="G110" s="5" t="inlineStr">
         <is>
           <t>อติกานต์ - ชนะชล</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="A109" s="2" t="inlineStr">
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>วันเสาร์ที่ 31 ตุลาคม 2569</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="30" customHeight="1">
-      <c r="A110" s="3" t="inlineStr">
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr">
+      <c r="C112" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D110" s="3" t="inlineStr">
+      <c r="D112" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E110" s="3" t="inlineStr">
+      <c r="E112" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F110" s="3" t="inlineStr">
+      <c r="F112" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G110" s="3" t="inlineStr">
+      <c r="G112" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
-        <is>
-          <t>15:30-18:30</t>
-        </is>
-      </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>126331</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>PSB1201</t>
-        </is>
-      </c>
-      <c r="E111" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="F111" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.อัจฉรา - วรินทร</t>
-        </is>
-      </c>
-      <c r="G111" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="4" t="inlineStr">
-        <is>
-          <t>15:30-18:30</t>
-        </is>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>127338</t>
-        </is>
-      </c>
-      <c r="C112" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>PSB1307</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.มานิตา - วีรภัทร์</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>พีชชา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4061,145 +4049,145 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
+          <t>126331</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>PSB1201</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.อัจฉรา - วรินทร</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>พีชชา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>127338</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>PSB1307</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>อ.ดร.มานิตา - วีรภัทร์</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>พีชชา - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
           <t>127432</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
         <is>
           <t>PSB1205</t>
         </is>
       </c>
-      <c r="E113" s="4" t="n">
+      <c r="E115" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="F113" s="5" t="inlineStr">
+      <c r="F115" s="5" t="inlineStr">
         <is>
           <t>ผศ.ดร.วันพัฒน์ - มาธวี</t>
         </is>
       </c>
-      <c r="G113" s="5" t="inlineStr">
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>พีชชา - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="2" t="inlineStr">
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>วันอาทิตย์ที่ 1 พฤศจิกายน 2569</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="30" customHeight="1">
-      <c r="A115" s="3" t="inlineStr">
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B117" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C115" s="3" t="inlineStr">
+      <c r="C117" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D115" s="3" t="inlineStr">
+      <c r="D117" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E115" s="3" t="inlineStr">
+      <c r="E117" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F115" s="3" t="inlineStr">
+      <c r="F117" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G115" s="3" t="inlineStr">
+      <c r="G117" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr">
-        <is>
-          <t>15:30-18:30</t>
-        </is>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>126218</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D116" s="4" t="inlineStr">
-        <is>
-          <t>PSB1101</t>
-        </is>
-      </c>
-      <c r="E116" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="F116" s="5" t="inlineStr">
-        <is>
-          <t>รศ.ดร.LEE - ณภัคสุรางค์</t>
-        </is>
-      </c>
-      <c r="G116" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
-        <is>
-          <t>15:30-18:30</t>
-        </is>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>126336</t>
-        </is>
-      </c>
-      <c r="C117" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D117" s="4" t="inlineStr">
-        <is>
-          <t>PSB1205</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="F117" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.กมลพร - สารัตถ์</t>
-        </is>
-      </c>
-      <c r="G117" s="5" t="inlineStr">
-        <is>
-          <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4199,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>126433</t>
+          <t>126218</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -4221,15 +4209,15 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>PSB1201</t>
+          <t>PSB1101</t>
         </is>
       </c>
       <c r="E118" s="4" t="n">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>อ.ดร.ศิรดา - วีรภัทร์</t>
+          <t>รศ.ดร.LEE - ณภัคสุรางค์</t>
         </is>
       </c>
       <c r="G118" s="5" t="inlineStr">
@@ -4246,7 +4234,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>127337</t>
+          <t>126336</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -4256,15 +4244,15 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>AUD50</t>
+          <t>PSB1205</t>
         </is>
       </c>
       <c r="E119" s="4" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.ภาณุวัฒน์ - ชัยตรี</t>
+          <t>ผศ.ดร.กมลพร - สารัตถ์</t>
         </is>
       </c>
       <c r="G119" s="5" t="inlineStr">
@@ -4281,7 +4269,7 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>127426</t>
+          <t>126433</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
@@ -4291,15 +4279,15 @@
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>PSB1204</t>
+          <t>PSB1201</t>
         </is>
       </c>
       <c r="E120" s="4" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>ผศ.ดร.สุพิชฌาย์ - อิสรีย์</t>
+          <t>อ.ดร.ศิรดา - วีรภัทร์</t>
         </is>
       </c>
       <c r="G120" s="5" t="inlineStr">
@@ -4316,7 +4304,7 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>128401</t>
+          <t>127337</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -4326,15 +4314,15 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>PSB1310</t>
+          <t>AUD50</t>
         </is>
       </c>
       <c r="E121" s="4" t="n">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>รศ.ดร.ธันยวัฒน์ - ณัฐธยาน์</t>
+          <t>ผศ.ดร.ภาณุวัฒน์ - ชัยตรี</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr">
@@ -4351,145 +4339,145 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
+          <t>127426</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>PSB1204</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.สุพิชฌาย์ - อิสรีย์</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
           <t>128401</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr">
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>PSB1310</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>รศ.ดร.ธันยวัฒน์ - ณัฐธยาน์</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>วรินทร - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>15:30-18:30</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>128401</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D124" s="4" t="inlineStr">
         <is>
           <t>PSB1302</t>
         </is>
       </c>
-      <c r="E122" s="4" t="n">
+      <c r="E124" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="F122" s="5" t="inlineStr">
+      <c r="F124" s="5" t="inlineStr">
         <is>
           <t>อ.พิกุล - ฐิตารีย์</t>
         </is>
       </c>
-      <c r="G122" s="5" t="inlineStr">
+      <c r="G124" s="5" t="inlineStr">
         <is>
           <t>วรินทร - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="20" customHeight="1">
-      <c r="A123" s="2" t="inlineStr">
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
         <is>
           <t>วันจันทร์ที่ 2 พฤศจิกายน 2569</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="30" customHeight="1">
-      <c r="A124" s="3" t="inlineStr">
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="3" t="inlineStr">
         <is>
           <t>เวลา</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="B126" s="3" t="inlineStr">
         <is>
           <t>วิชา</t>
         </is>
       </c>
-      <c r="C124" s="3" t="inlineStr">
+      <c r="C126" s="3" t="inlineStr">
         <is>
           <t>ตอน</t>
         </is>
       </c>
-      <c r="D124" s="3" t="inlineStr">
+      <c r="D126" s="3" t="inlineStr">
         <is>
           <t>ห้อง</t>
         </is>
       </c>
-      <c r="E124" s="3" t="inlineStr">
+      <c r="E126" s="3" t="inlineStr">
         <is>
           <t>นศ.</t>
         </is>
       </c>
-      <c r="F124" s="3" t="inlineStr">
+      <c r="F126" s="3" t="inlineStr">
         <is>
           <t>ผู้คุมสอบ
 (อาจารย์ - พนักงาน)</t>
         </is>
       </c>
-      <c r="G124" s="3" t="inlineStr">
+      <c r="G126" s="3" t="inlineStr">
         <is>
           <t>ผู้กระจายข้อสอบ - ผู้เปิดห้อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B125" s="4" t="inlineStr">
-        <is>
-          <t>127207</t>
-        </is>
-      </c>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D125" s="4" t="inlineStr">
-        <is>
-          <t>PSB1204</t>
-        </is>
-      </c>
-      <c r="E125" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="F125" s="5" t="inlineStr">
-        <is>
-          <t>ผศ.ดร.สุพิชฌาย์ - สกาวกวิน</t>
-        </is>
-      </c>
-      <c r="G125" s="5" t="inlineStr">
-        <is>
-          <t>มาธวี - ธีราภัณฑ์</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="4" t="inlineStr">
-        <is>
-          <t>08:00-11:00</t>
-        </is>
-      </c>
-      <c r="B126" s="4" t="inlineStr">
-        <is>
-          <t>127207</t>
-        </is>
-      </c>
-      <c r="C126" s="4" t="inlineStr">
-        <is>
-          <t>002</t>
-        </is>
-      </c>
-      <c r="D126" s="4" t="inlineStr">
-        <is>
-          <t>PSB1307</t>
-        </is>
-      </c>
-      <c r="E126" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="F126" s="5" t="inlineStr">
-        <is>
-          <t>อ.ดร.พินสุดา - วรินทร</t>
-        </is>
-      </c>
-      <c r="G126" s="5" t="inlineStr">
-        <is>
-          <t>มาธวี - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
@@ -4506,44 +4494,114 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>PSB1204</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>ผศ.ดร.สุพิชฌาย์ - สกาวกวิน</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>มาธวี - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>08:00-11:00</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>127207</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>PSB1307</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>อ.ดร.พินสุดา - วรินทร</t>
+        </is>
+      </c>
+      <c r="G128" s="5" t="inlineStr">
+        <is>
+          <t>มาธวี - ธีราภัณฑ์</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>08:00-11:00</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>127207</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
           <t>003</t>
         </is>
       </c>
-      <c r="D127" s="4" t="inlineStr">
+      <c r="D129" s="4" t="inlineStr">
         <is>
           <t>PSB1207</t>
         </is>
       </c>
-      <c r="E127" s="4" t="n">
+      <c r="E129" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="F127" s="5" t="inlineStr">
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>อ.ดร.มานิตา - พิชชารีย์</t>
         </is>
       </c>
-      <c r="G127" s="5" t="inlineStr">
+      <c r="G129" s="5" t="inlineStr">
         <is>
           <t>มาธวี - ธีราภัณฑ์</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="7" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
         <is>
           <t>หมายเหตุ (ยังต้องตัดสินใจ)</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="32" customHeight="1">
-      <c r="A130" s="8" t="inlineStr">
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="7" t="inlineStr">
         <is>
           <t>• ห้อง PSB1302 2026-10-22 12:00–15:00 นั่ง 54 คน จากความจุ 55 (ปกติใช้ 53 เผื่อไว้ 2) — กินที่เผื่อไป 1 ที่ ตามมติผู้ดูแล เพราะไม่มีห้องอื่นที่พอในช่วงนั้น</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="32" customHeight="1">
-      <c r="A131" s="8" t="inlineStr">
+    <row r="133" ht="32" customHeight="1">
+      <c r="A133" s="7" t="inlineStr">
         <is>
           <t>• คนคุมสอบไม่พอ 2026-10-27 12:00–15:00 ห้อง PSB1306 วิชา 126101 ตอน 004 ขาดอีก 1 คน</t>
         </is>
@@ -4551,23 +4609,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A123:G123"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A93:G93"/>
+    <mergeCell ref="A111:G111"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="A106:G106"/>
+    <mergeCell ref="A116:G116"/>
+    <mergeCell ref="A132:G132"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A91:G91"/>
-    <mergeCell ref="A69:G69"/>
-    <mergeCell ref="A109:G109"/>
-    <mergeCell ref="A114:G114"/>
-    <mergeCell ref="A131:G131"/>
-    <mergeCell ref="A101:G101"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A130:G130"/>
+    <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A125:G125"/>
+    <mergeCell ref="A103:G103"/>
+    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A133:G133"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>